<commit_message>
Update Unova routing to use letters for chains and populate missing families
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Unova_Path.xlsx
+++ b/Unova_Path.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F239"/>
+  <dimension ref="A1:F256"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6280,247 +6280,801 @@
         </is>
       </c>
       <c r="C226" t="inlineStr"/>
-      <c r="D226" t="inlineStr"/>
+      <c r="D226" t="inlineStr">
+        <is>
+          <t>Roggenrola</t>
+        </is>
+      </c>
       <c r="E226" t="inlineStr">
         <is>
           <t>76-78</t>
         </is>
       </c>
-      <c r="F226" t="inlineStr"/>
+      <c r="F226" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>Nature Sanctuary</t>
+          <t>Cave of Being</t>
         </is>
       </c>
       <c r="C227" t="inlineStr"/>
-      <c r="D227" t="inlineStr"/>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>Axew</t>
+        </is>
+      </c>
       <c r="E227" t="inlineStr">
         <is>
-          <t>78-80</t>
-        </is>
-      </c>
-      <c r="F227" t="inlineStr"/>
+          <t>76-78</t>
+        </is>
+      </c>
+      <c r="F227" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>Pinwheel Forest</t>
+          <t>Nature Sanctuary</t>
         </is>
       </c>
       <c r="C228" t="inlineStr"/>
-      <c r="D228" t="inlineStr"/>
+      <c r="D228" t="inlineStr">
+        <is>
+          <t>Yanma</t>
+        </is>
+      </c>
       <c r="E228" t="inlineStr">
         <is>
-          <t>80-81</t>
-        </is>
-      </c>
-      <c r="F228" t="inlineStr"/>
+          <t>78-80</t>
+        </is>
+      </c>
+      <c r="F228" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="n">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>Nacrene City</t>
+          <t>Nature Sanctuary</t>
         </is>
       </c>
       <c r="C229" t="inlineStr"/>
-      <c r="D229" t="inlineStr"/>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>Zorua</t>
+        </is>
+      </c>
       <c r="E229" t="inlineStr">
         <is>
-          <t>81-83</t>
-        </is>
-      </c>
-      <c r="F229" t="inlineStr"/>
+          <t>78-80</t>
+        </is>
+      </c>
+      <c r="F229" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>Moor of Icirrus</t>
+          <t>Pinwheel Forest</t>
         </is>
       </c>
       <c r="C230" t="inlineStr"/>
-      <c r="D230" t="inlineStr"/>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>Larvesta</t>
+        </is>
+      </c>
       <c r="E230" t="inlineStr">
         <is>
-          <t>83-85</t>
-        </is>
-      </c>
-      <c r="F230" t="inlineStr"/>
+          <t>80-81</t>
+        </is>
+      </c>
+      <c r="F230" t="inlineStr">
+        <is>
+          <t>33.34%</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>Icirrus City</t>
+          <t>Pinwheel Forest</t>
         </is>
       </c>
       <c r="C231" t="inlineStr"/>
-      <c r="D231" t="inlineStr"/>
+      <c r="D231" t="inlineStr">
+        <is>
+          <t>Snivy</t>
+        </is>
+      </c>
       <c r="E231" t="inlineStr">
         <is>
-          <t>85-86</t>
-        </is>
-      </c>
-      <c r="F231" t="inlineStr"/>
+          <t>80-81</t>
+        </is>
+      </c>
+      <c r="F231" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Striaton City</t>
+          <t>Pinwheel Forest</t>
         </is>
       </c>
       <c r="C232" t="inlineStr"/>
-      <c r="D232" t="inlineStr"/>
+      <c r="D232" t="inlineStr">
+        <is>
+          <t>Pansage</t>
+        </is>
+      </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>86-88</t>
-        </is>
-      </c>
-      <c r="F232" t="inlineStr"/>
+          <t>80-81</t>
+        </is>
+      </c>
+      <c r="F232" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="n">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>Dreamyard</t>
+          <t>Nacrene City</t>
         </is>
       </c>
       <c r="C233" t="inlineStr"/>
-      <c r="D233" t="inlineStr"/>
+      <c r="D233" t="inlineStr">
+        <is>
+          <t>Aron</t>
+        </is>
+      </c>
       <c r="E233" t="inlineStr">
         <is>
-          <t>88-90</t>
-        </is>
-      </c>
-      <c r="F233" t="inlineStr"/>
+          <t>81-83</t>
+        </is>
+      </c>
+      <c r="F233" t="inlineStr">
+        <is>
+          <t>33.34%</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Wellspring Cave</t>
+          <t>Nacrene City</t>
         </is>
       </c>
       <c r="C234" t="inlineStr"/>
-      <c r="D234" t="inlineStr"/>
+      <c r="D234" t="inlineStr">
+        <is>
+          <t>Tympole</t>
+        </is>
+      </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>90-91</t>
-        </is>
-      </c>
-      <c r="F234" t="inlineStr"/>
+          <t>81-83</t>
+        </is>
+      </c>
+      <c r="F234" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>P2 Laboratory</t>
+          <t>Nacrene City</t>
         </is>
       </c>
       <c r="C235" t="inlineStr"/>
-      <c r="D235" t="inlineStr"/>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>Budew</t>
+        </is>
+      </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>91-93</t>
-        </is>
-      </c>
-      <c r="F235" t="inlineStr"/>
+          <t>81-83</t>
+        </is>
+      </c>
+      <c r="F235" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Route 1</t>
+          <t>Moor of Icirrus</t>
         </is>
       </c>
       <c r="C236" t="inlineStr"/>
-      <c r="D236" t="inlineStr"/>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>Vullaby</t>
+        </is>
+      </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>93-95</t>
-        </is>
-      </c>
-      <c r="F236" t="inlineStr"/>
+          <t>83-85</t>
+        </is>
+      </c>
+      <c r="F236" t="inlineStr">
+        <is>
+          <t>33.34%</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Route 2</t>
+          <t>Moor of Icirrus</t>
         </is>
       </c>
       <c r="C237" t="inlineStr"/>
-      <c r="D237" t="inlineStr"/>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>Shelmet</t>
+        </is>
+      </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>95-96</t>
-        </is>
-      </c>
-      <c r="F237" t="inlineStr"/>
+          <t>83-85</t>
+        </is>
+      </c>
+      <c r="F237" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Route 3</t>
+          <t>Moor of Icirrus</t>
         </is>
       </c>
       <c r="C238" t="inlineStr"/>
-      <c r="D238" t="inlineStr"/>
+      <c r="D238" t="inlineStr">
+        <is>
+          <t>Ducklett</t>
+        </is>
+      </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>96-98</t>
-        </is>
-      </c>
-      <c r="F238" t="inlineStr"/>
+          <t>83-85</t>
+        </is>
+      </c>
+      <c r="F238" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
+        <v>49</v>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Icirrus City</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr"/>
+      <c r="D239" t="inlineStr">
+        <is>
+          <t>Lapras</t>
+        </is>
+      </c>
+      <c r="E239" t="inlineStr">
+        <is>
+          <t>85-86</t>
+        </is>
+      </c>
+      <c r="F239" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="n">
+        <v>49</v>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Icirrus City</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr"/>
+      <c r="D240" t="inlineStr">
+        <is>
+          <t>Tirtouga</t>
+        </is>
+      </c>
+      <c r="E240" t="inlineStr">
+        <is>
+          <t>85-86</t>
+        </is>
+      </c>
+      <c r="F240" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="n">
+        <v>50</v>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Striaton City</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr"/>
+      <c r="D241" t="inlineStr">
+        <is>
+          <t>Panpour</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>86-88</t>
+        </is>
+      </c>
+      <c r="F241" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="n">
+        <v>50</v>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Striaton City</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr"/>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>Pansear</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>86-88</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="n">
+        <v>51</v>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Dreamyard</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr"/>
+      <c r="D243" t="inlineStr">
+        <is>
+          <t>Munna</t>
+        </is>
+      </c>
+      <c r="E243" t="inlineStr">
+        <is>
+          <t>88-90</t>
+        </is>
+      </c>
+      <c r="F243" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="n">
+        <v>51</v>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Dreamyard</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr"/>
+      <c r="D244" t="inlineStr">
+        <is>
+          <t>Rufflet</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>88-90</t>
+        </is>
+      </c>
+      <c r="F244" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="n">
+        <v>52</v>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Wellspring Cave</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr"/>
+      <c r="D245" t="inlineStr">
+        <is>
+          <t>Grimer</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>90-91</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="n">
+        <v>52</v>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Wellspring Cave</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr"/>
+      <c r="D246" t="inlineStr">
+        <is>
+          <t>Bronzor</t>
+        </is>
+      </c>
+      <c r="E246" t="inlineStr">
+        <is>
+          <t>90-91</t>
+        </is>
+      </c>
+      <c r="F246" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="n">
+        <v>53</v>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>P2 Laboratory</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr"/>
+      <c r="D247" t="inlineStr">
+        <is>
+          <t>Beldum</t>
+        </is>
+      </c>
+      <c r="E247" t="inlineStr">
+        <is>
+          <t>91-93</t>
+        </is>
+      </c>
+      <c r="F247" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="n">
+        <v>53</v>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>P2 Laboratory</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr"/>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>Pawniard</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>91-93</t>
+        </is>
+      </c>
+      <c r="F248" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="n">
+        <v>54</v>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Route 1</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr"/>
+      <c r="D249" t="inlineStr">
+        <is>
+          <t>Tepig</t>
+        </is>
+      </c>
+      <c r="E249" t="inlineStr">
+        <is>
+          <t>93-95</t>
+        </is>
+      </c>
+      <c r="F249" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="n">
+        <v>54</v>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Route 1</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr"/>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>Oshawott</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>93-95</t>
+        </is>
+      </c>
+      <c r="F250" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="n">
+        <v>55</v>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Route 2</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr"/>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>Blitzle</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
+          <t>95-96</t>
+        </is>
+      </c>
+      <c r="F251" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="n">
+        <v>55</v>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Route 2</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr"/>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>Spoink</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
+          <t>95-96</t>
+        </is>
+      </c>
+      <c r="F252" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="n">
+        <v>56</v>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Route 3</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr"/>
+      <c r="D253" t="inlineStr">
+        <is>
+          <t>Throh</t>
+        </is>
+      </c>
+      <c r="E253" t="inlineStr">
+        <is>
+          <t>96-98</t>
+        </is>
+      </c>
+      <c r="F253" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="n">
+        <v>56</v>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Route 3</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr"/>
+      <c r="D254" t="inlineStr">
+        <is>
+          <t>Sawk</t>
+        </is>
+      </c>
+      <c r="E254" t="inlineStr">
+        <is>
+          <t>96-98</t>
+        </is>
+      </c>
+      <c r="F254" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="n">
         <v>57</v>
       </c>
-      <c r="B239" t="inlineStr">
+      <c r="B255" t="inlineStr">
         <is>
           <t>Nuvema Town</t>
         </is>
       </c>
-      <c r="C239" t="inlineStr"/>
-      <c r="D239" t="inlineStr"/>
-      <c r="E239" t="inlineStr">
+      <c r="C255" t="inlineStr"/>
+      <c r="D255" t="inlineStr">
+        <is>
+          <t>Cleffa</t>
+        </is>
+      </c>
+      <c r="E255" t="inlineStr">
         <is>
           <t>98-100</t>
         </is>
       </c>
-      <c r="F239" t="inlineStr"/>
+      <c r="F255" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="n">
+        <v>57</v>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Nuvema Town</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr"/>
+      <c r="D256" t="inlineStr">
+        <is>
+          <t>Igglybuff</t>
+        </is>
+      </c>
+      <c r="E256" t="inlineStr">
+        <is>
+          <t>98-100</t>
+        </is>
+      </c>
+      <c r="F256" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7151,7 +7705,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Extra Challenge 1$1</t>
+          <t>Extra Challenge A$1</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -7168,7 +7722,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Extra Challenge 1$2</t>
+          <t>Extra Challenge A$2</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -7185,7 +7739,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Extra Challenge 1$3</t>
+          <t>Extra Challenge A$3</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -7202,7 +7756,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Extra Challenge 1$4</t>
+          <t>Extra Challenge A$4</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -7219,7 +7773,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Extra Challenge 1$5</t>
+          <t>Extra Challenge A$5</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -7236,7 +7790,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Extra Challenge 2$1</t>
+          <t>Extra Challenge B$1</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -7253,7 +7807,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Extra Challenge 2$2</t>
+          <t>Extra Challenge B$2</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -7270,7 +7824,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Extra Challenge 2$3</t>
+          <t>Extra Challenge B$3</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -7287,7 +7841,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Extra Challenge 2$4</t>
+          <t>Extra Challenge B$4</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -7304,7 +7858,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Extra Challenge 3$1</t>
+          <t>Extra Challenge C$1</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -7321,7 +7875,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Extra Challenge 3$2</t>
+          <t>Extra Challenge C$2</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -7338,7 +7892,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Extra Challenge 3$3</t>
+          <t>Extra Challenge C$3</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -7355,7 +7909,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Extra Challenge 3$4</t>
+          <t>Extra Challenge C$4</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -7372,7 +7926,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Extra Challenge 4$1</t>
+          <t>Extra Challenge D$1</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -7389,7 +7943,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Extra Challenge 4$2</t>
+          <t>Extra Challenge D$2</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -7406,7 +7960,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Extra Challenge 4$3</t>
+          <t>Extra Challenge D$3</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -7423,7 +7977,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Extra Challenge 4$4</t>
+          <t>Extra Challenge D$4</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -7440,7 +7994,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Extra Challenge 5$1</t>
+          <t>Extra Challenge E$1</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -7457,7 +8011,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Extra Challenge 5$2</t>
+          <t>Extra Challenge E$2</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -7474,7 +8028,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Extra Challenge 5$3</t>
+          <t>Extra Challenge E$3</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -7491,7 +8045,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Extra Challenge 5$4</t>
+          <t>Extra Challenge E$4</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -7516,7 +8070,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D168"/>
+  <dimension ref="A1:D137"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7566,7 +8120,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Snivy</t>
+          <t>Servine</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -7576,183 +8130,183 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Servine</t>
+          <t>Pignite</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Fire / Fighting</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tepig</t>
+          <t>Emboar</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Fire / Fighting</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Pignite</t>
+          <t>Dewott</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Fire / Fighting</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Emboar</t>
+          <t>Samurott</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Fire / Fighting</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Oshawott</t>
+          <t>Unfezant</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Normal / Flying</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Dewott</t>
+          <t>Swadloon</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Bug / Grass</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Samurott</t>
+          <t>Leavanny</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Bug / Grass</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Unfezant</t>
+          <t>Sunflora</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Normal / Flying</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -7764,17 +8318,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Swadloon</t>
+          <t>Herdier</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bug / Grass</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -7786,39 +8340,39 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Leavanny</t>
+          <t>Stoutland</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Bug / Grass</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Sunflora</t>
+          <t>Flaaffy</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -7830,17 +8384,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Herdier</t>
+          <t>Ampharos</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -7852,39 +8406,39 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Stoutland</t>
+          <t>Azumarill</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Water / Fairy</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Flaaffy</t>
+          <t>Lucario</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Fighting / Steel</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -7896,39 +8450,39 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ampharos</t>
+          <t>Simisage</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Azumarill</t>
+          <t>Simisear</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Water / Fairy</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -7940,17 +8494,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Lucario</t>
+          <t>Simipour</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Fighting / Steel</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -7962,149 +8516,149 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Pansage</t>
+          <t>Whirlipede</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Bug / Poison</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Simisage</t>
+          <t>Scolipede</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Bug / Poison</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Pansear</t>
+          <t>Weezing</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Poison</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Simisear</t>
+          <t>Magneton</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Electric / Steel</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Panpour</t>
+          <t>Magnezone</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Electric / Steel</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Simipour</t>
+          <t>Arcanine</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Whirlipede</t>
+          <t>Magmar</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Bug / Poison</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -8116,39 +8670,39 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Scolipede</t>
+          <t>Magmortar</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Bug / Poison</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Weezing</t>
+          <t>Electabuzz</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Poison</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -8160,17 +8714,17 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Magneton</t>
+          <t>Electivire</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Electric / Steel</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -8182,39 +8736,39 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Magnezone</t>
+          <t>Crobat</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Electric / Steel</t>
+          <t>Poison / Flying</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Arcanine</t>
+          <t>Swoobat</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Psychic / Flying</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -8226,17 +8780,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Magmar</t>
+          <t>Gigalith</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Rock</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -8248,39 +8802,39 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Magmortar</t>
+          <t>Steelix</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Steel / Ground</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Electabuzz</t>
+          <t>Conkeldurr</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Fighting</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -8292,39 +8846,39 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Electivire</t>
+          <t>Musharna</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Crobat</t>
+          <t>Clefable</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Poison / Flying</t>
+          <t>Fairy</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -8336,39 +8890,39 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Grimer</t>
+          <t>Vaporeon</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Poison</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Swoobat</t>
+          <t>Jolteon</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Psychic / Flying</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -8380,39 +8934,39 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Roggenrola</t>
+          <t>Flareon</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Rock</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Gigalith</t>
+          <t>Espeon</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Rock</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -8424,17 +8978,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Steelix</t>
+          <t>Umbreon</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Steel / Ground</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -8446,17 +9000,17 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Conkeldurr</t>
+          <t>Leafeon</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Fighting</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -8468,78 +9022,78 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Munna</t>
+          <t>Glaceon</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Musharna</t>
+          <t>Krokorok</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Ground / Dark</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cleffa</t>
+          <t>Krookodile</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Fairy</t>
+          <t>Ground / Dark</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Clefable</t>
+          <t>Darmanitan</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Fairy</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -8549,24 +9103,24 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Vaporeon</t>
+          <t>Cinccino</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -8578,17 +9132,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Jolteon</t>
+          <t>Sandslash</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Ground</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -8600,17 +9154,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Flareon</t>
+          <t>Scrafty</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Dark / Fighting</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -8622,17 +9176,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Espeon</t>
+          <t>Vibrava</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Ground / Dragon</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -8644,17 +9198,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Umbreon</t>
+          <t>Flygon</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Dark</t>
+          <t>Ground / Dragon</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -8666,17 +9220,17 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Leafeon</t>
+          <t>Cofagrigus</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Ghost</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -8688,17 +9242,17 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Glaceon</t>
+          <t>Carracosta</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Water / Rock</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -8710,12 +9264,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Krokorok</t>
+          <t>Archen</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Ground / Dark</t>
+          <t>Rock / Flying</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -8725,19 +9279,19 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Krookodile</t>
+          <t>Archeops</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ground / Dark</t>
+          <t>Rock / Flying</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -8754,17 +9308,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Darmanitan</t>
+          <t>Klang</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -8776,17 +9330,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Cinccino</t>
+          <t>Klinklang</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Steel</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -8798,61 +9352,61 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Rufflet</t>
+          <t>Vespiquen</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Normal / Flying</t>
+          <t>Bug / Flying</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Vullaby</t>
+          <t>Zoroark</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Dark / Flying</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Sandslash</t>
+          <t>Swanna</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ground</t>
+          <t>Water / Flying</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -8864,17 +9418,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Scrafty</t>
+          <t>Escavalier</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Dark / Fighting</t>
+          <t>Bug / Steel</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -8886,17 +9440,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Vibrava</t>
+          <t>Accelgor</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Ground / Dragon</t>
+          <t>Bug</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -8908,34 +9462,34 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Flygon</t>
+          <t>Sawsbuck</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Ground / Dragon</t>
+          <t>Normal / Grass</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Cofagrigus</t>
+          <t>Castform</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Ghost</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -8945,63 +9499,63 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Tirtouga</t>
+          <t>Probopass</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Water / Rock</t>
+          <t>Rock / Steel</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Carracosta</t>
+          <t>Aggron</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Water / Rock</t>
+          <t>Steel / Rock</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Archen</t>
+          <t>Baltoy</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Rock / Flying</t>
+          <t>Ground / Psychic</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -9018,12 +9572,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Archeops</t>
+          <t>Claydol</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Rock / Flying</t>
+          <t>Ground / Psychic</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -9040,17 +9594,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Klang</t>
+          <t>Volcarona</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Bug / Fire</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -9062,61 +9616,61 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Klinklang</t>
+          <t>Galvantula</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Steel</t>
+          <t>Bug / Electric</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Budew</t>
+          <t>Ferrothorn</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Grass / Poison</t>
+          <t>Grass / Steel</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Vespiquen</t>
+          <t>Eelektross</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Bug / Flying</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -9128,56 +9682,56 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Blitzle</t>
+          <t>Fraxure</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Dragon</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Zorua</t>
+          <t>Haxorus</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dark</t>
+          <t>Dragon</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Zoroark</t>
+          <t>Zangoose</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Dark</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -9194,12 +9748,12 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Ducklett</t>
+          <t>Seviper</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Water / Flying</t>
+          <t>Poison</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -9216,39 +9770,39 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Swanna</t>
+          <t>Beheeyem</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Water / Flying</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Escavalier</t>
+          <t>Lampent</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Bug / Steel</t>
+          <t>Ghost / Fire</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -9260,56 +9814,56 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Shelmet</t>
+          <t>Chandelure</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Ghost / Fire</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Accelgor</t>
+          <t>Beartic</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Bug</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Sawsbuck</t>
+          <t>Tornadus</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Normal / Grass</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -9319,19 +9873,19 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Castform</t>
+          <t>Thundurus</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -9348,12 +9902,12 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Probopass</t>
+          <t>Landorus</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Rock / Steel</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -9363,19 +9917,19 @@
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Skorupi</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Steel / Rock</t>
+          <t>Poison / Bug</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -9392,12 +9946,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Aggron</t>
+          <t>Drapion</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Steel / Rock</t>
+          <t>Poison / Dark</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -9407,19 +9961,19 @@
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Baltoy</t>
+          <t>Numel</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Ground / Psychic</t>
+          <t>Fire / Ground</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -9436,34 +9990,34 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Claydol</t>
+          <t>Grumpig</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Ground / Psychic</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Larvesta</t>
+          <t>Drifloon</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Bug / Fire</t>
+          <t>Ghost / Flying</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -9480,12 +10034,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Volcarona</t>
+          <t>Shuppet</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Bug / Fire</t>
+          <t>Ghost</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -9502,12 +10056,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Galvantula</t>
+          <t>Lunatone</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Bug / Electric</t>
+          <t>Rock / Psychic</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -9517,19 +10071,19 @@
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Ferrothorn</t>
+          <t>Solrock</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Grass / Steel</t>
+          <t>Rock / Psychic</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -9539,24 +10093,24 @@
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Eelektross</t>
+          <t>Tangrowth</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -9568,78 +10122,78 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Axew</t>
+          <t>Mienshao</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Dragon</t>
+          <t>Fighting</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Fraxure</t>
+          <t>Gliscor</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Dragon</t>
+          <t>Ground / Flying</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Haxorus</t>
+          <t>Bisharp</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Dragon</t>
+          <t>Dark / Steel</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Zangoose</t>
+          <t>Cobalion</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Steel / Fighting</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -9656,12 +10210,12 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Seviper</t>
+          <t>Terrakion</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Poison</t>
+          <t>Rock / Fighting</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -9678,12 +10232,12 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Beheeyem</t>
+          <t>Virizion</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Grass / Fighting</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -9693,24 +10247,24 @@
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Lampent</t>
+          <t>Seismitoad</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Ghost / Fire</t>
+          <t>Water / Ground</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -9722,12 +10276,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Chandelure</t>
+          <t>Shuckle</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Ghost / Fire</t>
+          <t>Bug / Rock</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -9744,17 +10298,17 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Beartic</t>
+          <t>Mantine</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Water / Flying</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
@@ -9766,17 +10320,17 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Tornadus</t>
+          <t>Octillery</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -9788,17 +10342,17 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Thundurus</t>
+          <t>Starmie</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Water / Psychic</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -9810,12 +10364,12 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Landorus</t>
+          <t>Wailmer</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -9825,19 +10379,19 @@
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Skorupi</t>
+          <t>Wailord</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Poison / Bug</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -9854,193 +10408,193 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Drapion</t>
+          <t>Sealeo</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Poison / Dark</t>
+          <t>Ice / Water</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Numel</t>
+          <t>Walrein</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Fire / Ground</t>
+          <t>Ice / Water</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Spoink</t>
+          <t>Ninetales</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Grumpig</t>
+          <t>Weavile</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Dark / Ice</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Drifloon</t>
+          <t>Vanillish</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Ghost / Flying</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Shuppet</t>
+          <t>Vanilluxe</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Ghost</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Lunatone</t>
+          <t>Mamoswine</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Rock / Psychic</t>
+          <t>Ice / Ground</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Solrock</t>
+          <t>Metagross</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Rock / Psychic</t>
+          <t>Steel / Psychic</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Tangrowth</t>
+          <t>Dewgong</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Water / Ice</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -10052,17 +10606,17 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Mienshao</t>
+          <t>Golurk</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Fighting</t>
+          <t>Ground / Ghost</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
@@ -10074,17 +10628,17 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Gliscor</t>
+          <t>Zweilous</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Ground / Flying</t>
+          <t>Dark / Dragon</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -10096,34 +10650,34 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Pawniard</t>
+          <t>Hydreigon</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Dark / Steel</t>
+          <t>Dark / Dragon</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Bisharp</t>
+          <t>Slakoth</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Dark / Steel</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -10140,12 +10694,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Cobalion</t>
+          <t>Vigoroth</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Steel / Fighting</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -10162,12 +10716,12 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Terrakion</t>
+          <t>Slaking</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Rock / Fighting</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -10184,61 +10738,61 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Virizion</t>
+          <t>Crawdaunt</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Grass / Fighting</t>
+          <t>Water / Dark</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Tympole</t>
+          <t>Jigglypuff</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Normal / Fairy</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Seismitoad</t>
+          <t>Wigglytuff</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Water / Ground</t>
+          <t>Normal / Fairy</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
@@ -10250,12 +10804,12 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Shuckle</t>
+          <t>Lickitung</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Bug / Rock</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -10272,12 +10826,12 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Mantine</t>
+          <t>Lickilicky</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Water / Flying</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -10287,24 +10841,24 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Octillery</t>
+          <t>Yanmega</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Bug / Flying</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -10316,12 +10870,12 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Starmie</t>
+          <t>Tropius</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Water / Psychic</t>
+          <t>Grass / Flying</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -10331,41 +10885,41 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Wailmer</t>
+          <t>Toxicroak</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Poison / Fighting</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Wailord</t>
+          <t>Larvitar</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Rock / Ground</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -10382,34 +10936,34 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Lapras</t>
+          <t>Tyranitar</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Water / Ice</t>
+          <t>Rock / Dark</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Sealeo</t>
+          <t>Reshiram</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Ice / Water</t>
+          <t>Dragon / Fire</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -10419,19 +10973,19 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Walrein</t>
+          <t>Zekrom</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Ice / Water</t>
+          <t>Dragon / Electric</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -10448,12 +11002,12 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Ninetales</t>
+          <t>Kyurem</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Dragon / Ice</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -10463,19 +11017,19 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Bronzor</t>
+          <t>Keldeo</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Steel / Psychic</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -10492,12 +11046,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>Weavile</t>
+          <t>Meloetta</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Dark / Ice</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -10507,19 +11061,19 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Vanillish</t>
+          <t>Genesect</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Bug / Steel</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -10528,688 +11082,6 @@
         </is>
       </c>
       <c r="D137" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="138">
-      <c r="A138" t="inlineStr">
-        <is>
-          <t>Vanilluxe</t>
-        </is>
-      </c>
-      <c r="B138" t="inlineStr">
-        <is>
-          <t>Ice</t>
-        </is>
-      </c>
-      <c r="C138" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D138" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>Mamoswine</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>Ice / Ground</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>Beldum</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>Steel / Psychic</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>Metagross</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Steel / Psychic</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>Dewgong</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Water / Ice</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>Throh</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>Fighting</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>Sawk</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>Fighting</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="145">
-      <c r="A145" t="inlineStr">
-        <is>
-          <t>Golurk</t>
-        </is>
-      </c>
-      <c r="B145" t="inlineStr">
-        <is>
-          <t>Ground / Ghost</t>
-        </is>
-      </c>
-      <c r="C145" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D145" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="146">
-      <c r="A146" t="inlineStr">
-        <is>
-          <t>Zweilous</t>
-        </is>
-      </c>
-      <c r="B146" t="inlineStr">
-        <is>
-          <t>Dark / Dragon</t>
-        </is>
-      </c>
-      <c r="C146" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D146" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="147">
-      <c r="A147" t="inlineStr">
-        <is>
-          <t>Hydreigon</t>
-        </is>
-      </c>
-      <c r="B147" t="inlineStr">
-        <is>
-          <t>Dark / Dragon</t>
-        </is>
-      </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D147" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="148">
-      <c r="A148" t="inlineStr">
-        <is>
-          <t>Slakoth</t>
-        </is>
-      </c>
-      <c r="B148" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="C148" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D148" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>Vigoroth</t>
-        </is>
-      </c>
-      <c r="B149" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="C149" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D149" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>Slaking</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="151">
-      <c r="A151" t="inlineStr">
-        <is>
-          <t>Crawdaunt</t>
-        </is>
-      </c>
-      <c r="B151" t="inlineStr">
-        <is>
-          <t>Water / Dark</t>
-        </is>
-      </c>
-      <c r="C151" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D151" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="152">
-      <c r="A152" t="inlineStr">
-        <is>
-          <t>Igglybuff</t>
-        </is>
-      </c>
-      <c r="B152" t="inlineStr">
-        <is>
-          <t>Normal / Fairy</t>
-        </is>
-      </c>
-      <c r="C152" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D152" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="153">
-      <c r="A153" t="inlineStr">
-        <is>
-          <t>Jigglypuff</t>
-        </is>
-      </c>
-      <c r="B153" t="inlineStr">
-        <is>
-          <t>Normal / Fairy</t>
-        </is>
-      </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D153" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>Wigglytuff</t>
-        </is>
-      </c>
-      <c r="B154" t="inlineStr">
-        <is>
-          <t>Normal / Fairy</t>
-        </is>
-      </c>
-      <c r="C154" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D154" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>Lickitung</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>Lickilicky</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>Normal</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>Yanma</t>
-        </is>
-      </c>
-      <c r="B157" t="inlineStr">
-        <is>
-          <t>Bug / Flying</t>
-        </is>
-      </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D157" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>Yanmega</t>
-        </is>
-      </c>
-      <c r="B158" t="inlineStr">
-        <is>
-          <t>Bug / Flying</t>
-        </is>
-      </c>
-      <c r="C158" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D158" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>Tropius</t>
-        </is>
-      </c>
-      <c r="B159" t="inlineStr">
-        <is>
-          <t>Grass / Flying</t>
-        </is>
-      </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D159" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>Toxicroak</t>
-        </is>
-      </c>
-      <c r="B160" t="inlineStr">
-        <is>
-          <t>Poison / Fighting</t>
-        </is>
-      </c>
-      <c r="C160" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D160" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>Larvitar</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>Rock / Ground</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>Tyranitar</t>
-        </is>
-      </c>
-      <c r="B162" t="inlineStr">
-        <is>
-          <t>Rock / Dark</t>
-        </is>
-      </c>
-      <c r="C162" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D162" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>Reshiram</t>
-        </is>
-      </c>
-      <c r="B163" t="inlineStr">
-        <is>
-          <t>Dragon / Fire</t>
-        </is>
-      </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D163" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>Zekrom</t>
-        </is>
-      </c>
-      <c r="B164" t="inlineStr">
-        <is>
-          <t>Dragon / Electric</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D164" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>Kyurem</t>
-        </is>
-      </c>
-      <c r="B165" t="inlineStr">
-        <is>
-          <t>Dragon / Ice</t>
-        </is>
-      </c>
-      <c r="C165" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D165" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>Keldeo</t>
-        </is>
-      </c>
-      <c r="B166" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D166" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>Meloetta</t>
-        </is>
-      </c>
-      <c r="B167" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C167" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D167" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>Genesect</t>
-        </is>
-      </c>
-      <c r="B168" t="inlineStr">
-        <is>
-          <t>Bug / Steel</t>
-        </is>
-      </c>
-      <c r="C168" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D168" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Update Unova paths to include leveled legendaries at end of challenge chains
Co-authored-by: lsampaio1337-beep <246645260+lsampaio1337-beep@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Unova_Path.xlsx
+++ b/Unova_Path.xlsx
@@ -415,7 +415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F256"/>
+  <dimension ref="A1:F266"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6386,7 +6386,7 @@
       <c r="C230" t="inlineStr"/>
       <c r="D230" t="inlineStr">
         <is>
-          <t>Larvesta</t>
+          <t>Snivy</t>
         </is>
       </c>
       <c r="E230" t="inlineStr">
@@ -6396,7 +6396,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t>33.34%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -6412,7 +6412,7 @@
       <c r="C231" t="inlineStr"/>
       <c r="D231" t="inlineStr">
         <is>
-          <t>Snivy</t>
+          <t>Pansage</t>
         </is>
       </c>
       <c r="E231" t="inlineStr">
@@ -6422,33 +6422,33 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>Pinwheel Forest</t>
+          <t>Nacrene City</t>
         </is>
       </c>
       <c r="C232" t="inlineStr"/>
       <c r="D232" t="inlineStr">
         <is>
-          <t>Pansage</t>
+          <t>Tympole</t>
         </is>
       </c>
       <c r="E232" t="inlineStr">
         <is>
-          <t>80-81</t>
+          <t>81-83</t>
         </is>
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -6464,7 +6464,7 @@
       <c r="C233" t="inlineStr"/>
       <c r="D233" t="inlineStr">
         <is>
-          <t>Aron</t>
+          <t>Budew</t>
         </is>
       </c>
       <c r="E233" t="inlineStr">
@@ -6474,158 +6474,158 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t>33.34%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B234" t="inlineStr">
         <is>
-          <t>Nacrene City</t>
+          <t>Moor of Icirrus</t>
         </is>
       </c>
       <c r="C234" t="inlineStr"/>
       <c r="D234" t="inlineStr">
         <is>
-          <t>Tympole</t>
+          <t>Shelmet</t>
         </is>
       </c>
       <c r="E234" t="inlineStr">
         <is>
-          <t>81-83</t>
+          <t>83-85</t>
         </is>
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B235" t="inlineStr">
         <is>
-          <t>Nacrene City</t>
+          <t>Moor of Icirrus</t>
         </is>
       </c>
       <c r="C235" t="inlineStr"/>
       <c r="D235" t="inlineStr">
         <is>
-          <t>Budew</t>
+          <t>Ducklett</t>
         </is>
       </c>
       <c r="E235" t="inlineStr">
         <is>
-          <t>81-83</t>
+          <t>83-85</t>
         </is>
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B236" t="inlineStr">
         <is>
-          <t>Moor of Icirrus</t>
+          <t>Icirrus City</t>
         </is>
       </c>
       <c r="C236" t="inlineStr"/>
       <c r="D236" t="inlineStr">
         <is>
-          <t>Vullaby</t>
+          <t>Lapras</t>
         </is>
       </c>
       <c r="E236" t="inlineStr">
         <is>
-          <t>83-85</t>
+          <t>85-86</t>
         </is>
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>33.34%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B237" t="inlineStr">
         <is>
-          <t>Moor of Icirrus</t>
+          <t>Icirrus City</t>
         </is>
       </c>
       <c r="C237" t="inlineStr"/>
       <c r="D237" t="inlineStr">
         <is>
-          <t>Shelmet</t>
+          <t>Tirtouga</t>
         </is>
       </c>
       <c r="E237" t="inlineStr">
         <is>
-          <t>83-85</t>
+          <t>85-86</t>
         </is>
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="B238" t="inlineStr">
         <is>
-          <t>Moor of Icirrus</t>
+          <t>Striaton City</t>
         </is>
       </c>
       <c r="C238" t="inlineStr"/>
       <c r="D238" t="inlineStr">
         <is>
-          <t>Ducklett</t>
+          <t>Panpour</t>
         </is>
       </c>
       <c r="E238" t="inlineStr">
         <is>
-          <t>83-85</t>
+          <t>86-88</t>
         </is>
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>33.33%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B239" t="inlineStr">
         <is>
-          <t>Icirrus City</t>
+          <t>Striaton City</t>
         </is>
       </c>
       <c r="C239" t="inlineStr"/>
       <c r="D239" t="inlineStr">
         <is>
-          <t>Lapras</t>
+          <t>Pansear</t>
         </is>
       </c>
       <c r="E239" t="inlineStr">
         <is>
-          <t>85-86</t>
+          <t>86-88</t>
         </is>
       </c>
       <c r="F239" t="inlineStr">
@@ -6636,22 +6636,22 @@
     </row>
     <row r="240">
       <c r="A240" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B240" t="inlineStr">
         <is>
-          <t>Icirrus City</t>
+          <t>Dreamyard</t>
         </is>
       </c>
       <c r="C240" t="inlineStr"/>
       <c r="D240" t="inlineStr">
         <is>
-          <t>Tirtouga</t>
+          <t>Munna</t>
         </is>
       </c>
       <c r="E240" t="inlineStr">
         <is>
-          <t>85-86</t>
+          <t>88-90</t>
         </is>
       </c>
       <c r="F240" t="inlineStr">
@@ -6662,22 +6662,22 @@
     </row>
     <row r="241">
       <c r="A241" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B241" t="inlineStr">
         <is>
-          <t>Striaton City</t>
+          <t>Dreamyard</t>
         </is>
       </c>
       <c r="C241" t="inlineStr"/>
       <c r="D241" t="inlineStr">
         <is>
-          <t>Panpour</t>
+          <t>Rufflet</t>
         </is>
       </c>
       <c r="E241" t="inlineStr">
         <is>
-          <t>86-88</t>
+          <t>88-90</t>
         </is>
       </c>
       <c r="F241" t="inlineStr">
@@ -6688,22 +6688,22 @@
     </row>
     <row r="242">
       <c r="A242" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>Striaton City</t>
+          <t>Wellspring Cave</t>
         </is>
       </c>
       <c r="C242" t="inlineStr"/>
       <c r="D242" t="inlineStr">
         <is>
-          <t>Pansear</t>
+          <t>Grimer</t>
         </is>
       </c>
       <c r="E242" t="inlineStr">
         <is>
-          <t>86-88</t>
+          <t>90-91</t>
         </is>
       </c>
       <c r="F242" t="inlineStr">
@@ -6714,22 +6714,22 @@
     </row>
     <row r="243">
       <c r="A243" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>Dreamyard</t>
+          <t>Wellspring Cave</t>
         </is>
       </c>
       <c r="C243" t="inlineStr"/>
       <c r="D243" t="inlineStr">
         <is>
-          <t>Munna</t>
+          <t>Bronzor</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>88-90</t>
+          <t>90-91</t>
         </is>
       </c>
       <c r="F243" t="inlineStr">
@@ -6740,22 +6740,22 @@
     </row>
     <row r="244">
       <c r="A244" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Dreamyard</t>
+          <t>P2 Laboratory</t>
         </is>
       </c>
       <c r="C244" t="inlineStr"/>
       <c r="D244" t="inlineStr">
         <is>
-          <t>Rufflet</t>
+          <t>Beldum</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
         <is>
-          <t>88-90</t>
+          <t>91-93</t>
         </is>
       </c>
       <c r="F244" t="inlineStr">
@@ -6766,22 +6766,22 @@
     </row>
     <row r="245">
       <c r="A245" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Wellspring Cave</t>
+          <t>P2 Laboratory</t>
         </is>
       </c>
       <c r="C245" t="inlineStr"/>
       <c r="D245" t="inlineStr">
         <is>
-          <t>Grimer</t>
+          <t>Pawniard</t>
         </is>
       </c>
       <c r="E245" t="inlineStr">
         <is>
-          <t>90-91</t>
+          <t>91-93</t>
         </is>
       </c>
       <c r="F245" t="inlineStr">
@@ -6792,22 +6792,22 @@
     </row>
     <row r="246">
       <c r="A246" t="n">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Wellspring Cave</t>
+          <t>Route 1</t>
         </is>
       </c>
       <c r="C246" t="inlineStr"/>
       <c r="D246" t="inlineStr">
         <is>
-          <t>Bronzor</t>
+          <t>Tepig</t>
         </is>
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>90-91</t>
+          <t>93-95</t>
         </is>
       </c>
       <c r="F246" t="inlineStr">
@@ -6818,22 +6818,22 @@
     </row>
     <row r="247">
       <c r="A247" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>P2 Laboratory</t>
+          <t>Route 1</t>
         </is>
       </c>
       <c r="C247" t="inlineStr"/>
       <c r="D247" t="inlineStr">
         <is>
-          <t>Beldum</t>
+          <t>Oshawott</t>
         </is>
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>91-93</t>
+          <t>93-95</t>
         </is>
       </c>
       <c r="F247" t="inlineStr">
@@ -6844,22 +6844,22 @@
     </row>
     <row r="248">
       <c r="A248" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>P2 Laboratory</t>
+          <t>Route 2</t>
         </is>
       </c>
       <c r="C248" t="inlineStr"/>
       <c r="D248" t="inlineStr">
         <is>
-          <t>Pawniard</t>
+          <t>Blitzle</t>
         </is>
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>91-93</t>
+          <t>95-96</t>
         </is>
       </c>
       <c r="F248" t="inlineStr">
@@ -6870,22 +6870,22 @@
     </row>
     <row r="249">
       <c r="A249" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Route 1</t>
+          <t>Route 2</t>
         </is>
       </c>
       <c r="C249" t="inlineStr"/>
       <c r="D249" t="inlineStr">
         <is>
-          <t>Tepig</t>
+          <t>Spoink</t>
         </is>
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>93-95</t>
+          <t>95-96</t>
         </is>
       </c>
       <c r="F249" t="inlineStr">
@@ -6896,22 +6896,22 @@
     </row>
     <row r="250">
       <c r="A250" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Route 1</t>
+          <t>Route 3</t>
         </is>
       </c>
       <c r="C250" t="inlineStr"/>
       <c r="D250" t="inlineStr">
         <is>
-          <t>Oshawott</t>
+          <t>Throh</t>
         </is>
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>93-95</t>
+          <t>96-98</t>
         </is>
       </c>
       <c r="F250" t="inlineStr">
@@ -6922,22 +6922,22 @@
     </row>
     <row r="251">
       <c r="A251" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Route 2</t>
+          <t>Route 3</t>
         </is>
       </c>
       <c r="C251" t="inlineStr"/>
       <c r="D251" t="inlineStr">
         <is>
-          <t>Blitzle</t>
+          <t>Sawk</t>
         </is>
       </c>
       <c r="E251" t="inlineStr">
         <is>
-          <t>95-96</t>
+          <t>96-98</t>
         </is>
       </c>
       <c r="F251" t="inlineStr">
@@ -6948,22 +6948,22 @@
     </row>
     <row r="252">
       <c r="A252" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Route 2</t>
+          <t>Nuvema Town</t>
         </is>
       </c>
       <c r="C252" t="inlineStr"/>
       <c r="D252" t="inlineStr">
         <is>
-          <t>Spoink</t>
+          <t>Cleffa</t>
         </is>
       </c>
       <c r="E252" t="inlineStr">
         <is>
-          <t>95-96</t>
+          <t>98-100</t>
         </is>
       </c>
       <c r="F252" t="inlineStr">
@@ -6974,22 +6974,22 @@
     </row>
     <row r="253">
       <c r="A253" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Route 3</t>
+          <t>Nuvema Town</t>
         </is>
       </c>
       <c r="C253" t="inlineStr"/>
       <c r="D253" t="inlineStr">
         <is>
-          <t>Throh</t>
+          <t>Igglybuff</t>
         </is>
       </c>
       <c r="E253" t="inlineStr">
         <is>
-          <t>96-98</t>
+          <t>98-100</t>
         </is>
       </c>
       <c r="F253" t="inlineStr">
@@ -7000,79 +7000,339 @@
     </row>
     <row r="254">
       <c r="A254" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Route 3</t>
+          <t>Moor of Icirrus Depths</t>
         </is>
       </c>
       <c r="C254" t="inlineStr"/>
       <c r="D254" t="inlineStr">
         <is>
-          <t>Sawk</t>
+          <t>Cobalion</t>
         </is>
       </c>
       <c r="E254" t="inlineStr">
         <is>
-          <t>96-98</t>
+          <t>110</t>
         </is>
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Nuvema Town</t>
+          <t>Moor of Icirrus Depths</t>
         </is>
       </c>
       <c r="C255" t="inlineStr"/>
       <c r="D255" t="inlineStr">
         <is>
-          <t>Cleffa</t>
+          <t>Terrakion</t>
         </is>
       </c>
       <c r="E255" t="inlineStr">
         <is>
-          <t>98-100</t>
+          <t>110</t>
         </is>
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>25.0%</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Nuvema Town</t>
+          <t>Moor of Icirrus Depths</t>
         </is>
       </c>
       <c r="C256" t="inlineStr"/>
       <c r="D256" t="inlineStr">
         <is>
-          <t>Igglybuff</t>
+          <t>Virizion</t>
         </is>
       </c>
       <c r="E256" t="inlineStr">
         <is>
-          <t>98-100</t>
+          <t>110</t>
         </is>
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>25.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="n">
+        <v>58</v>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Moor of Icirrus Depths</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr"/>
+      <c r="D257" t="inlineStr">
+        <is>
+          <t>Keldeo</t>
+        </is>
+      </c>
+      <c r="E257" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="F257" t="inlineStr">
+        <is>
+          <t>25.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="n">
+        <v>59</v>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Liberty Garden</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr"/>
+      <c r="D258" t="inlineStr">
+        <is>
+          <t>Victini</t>
+        </is>
+      </c>
+      <c r="E258" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="F258" t="inlineStr">
+        <is>
+          <t>33.34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="n">
+        <v>59</v>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Liberty Garden</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr"/>
+      <c r="D259" t="inlineStr">
+        <is>
+          <t>Meloetta</t>
+        </is>
+      </c>
+      <c r="E259" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="F259" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="n">
+        <v>59</v>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Liberty Garden</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr"/>
+      <c r="D260" t="inlineStr">
+        <is>
+          <t>Genesect</t>
+        </is>
+      </c>
+      <c r="E260" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="F260" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="n">
+        <v>60</v>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Abundant Shrine Depths</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr"/>
+      <c r="D261" t="inlineStr">
+        <is>
+          <t>Landorus</t>
+        </is>
+      </c>
+      <c r="E261" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="F261" t="inlineStr">
+        <is>
+          <t>33.34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="n">
+        <v>60</v>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Abundant Shrine Depths</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr"/>
+      <c r="D262" t="inlineStr">
+        <is>
+          <t>Thundurus</t>
+        </is>
+      </c>
+      <c r="E262" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="F262" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="n">
+        <v>60</v>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Abundant Shrine Depths</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr"/>
+      <c r="D263" t="inlineStr">
+        <is>
+          <t>Tornadus</t>
+        </is>
+      </c>
+      <c r="E263" t="inlineStr">
+        <is>
+          <t>110</t>
+        </is>
+      </c>
+      <c r="F263" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="n">
+        <v>61</v>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>N's Castle</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr"/>
+      <c r="D264" t="inlineStr">
+        <is>
+          <t>Kyurem</t>
+        </is>
+      </c>
+      <c r="E264" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F264" t="inlineStr">
+        <is>
+          <t>33.34%</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="n">
+        <v>61</v>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>N's Castle</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr"/>
+      <c r="D265" t="inlineStr">
+        <is>
+          <t>Reshiram</t>
+        </is>
+      </c>
+      <c r="E265" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F265" t="inlineStr">
+        <is>
+          <t>33.33%</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="n">
+        <v>61</v>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>N's Castle</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr"/>
+      <c r="D266" t="inlineStr">
+        <is>
+          <t>Zekrom</t>
+        </is>
+      </c>
+      <c r="E266" t="inlineStr">
+        <is>
+          <t>120</t>
+        </is>
+      </c>
+      <c r="F266" t="inlineStr">
+        <is>
+          <t>33.33%</t>
         </is>
       </c>
     </row>
@@ -7087,7 +7347,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C57"/>
+  <dimension ref="A1:C61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7926,136 +8186,204 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Extra Challenge D$1</t>
+          <t>Extra Challenge C$5</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Complete Challenge 35</t>
+          <t>Catch 10 Pokemon in Icirrus City</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Unlock Striaton City</t>
+          <t>Unlock Moor of Icirrus Depths</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Extra Challenge D$2</t>
+          <t>Extra Challenge D$1</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Catch 10 Pokemon in Striaton City</t>
+          <t>Complete Challenge 35</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Unlock Dreamyard</t>
+          <t>Unlock Striaton City</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Extra Challenge D$3</t>
+          <t>Extra Challenge D$2</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Catch 10 Pokemon in Dreamyard</t>
+          <t>Catch 10 Pokemon in Striaton City</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Unlock Wellspring Cave</t>
+          <t>Unlock Dreamyard</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Extra Challenge D$4</t>
+          <t>Extra Challenge D$3</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Catch 10 Pokemon in Wellspring Cave</t>
+          <t>Catch 10 Pokemon in Dreamyard</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Unlock P2 Laboratory</t>
+          <t>Unlock Wellspring Cave</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Extra Challenge E$1</t>
+          <t>Extra Challenge D$4</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Complete Challenge 35</t>
+          <t>Catch 10 Pokemon in Wellspring Cave</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Unlock Route 1</t>
+          <t>Unlock P2 Laboratory</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Extra Challenge E$2</t>
+          <t>Extra Challenge D$5</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Catch 10 Pokemon in Route 1</t>
+          <t>Catch 10 Pokemon in P2 Laboratory</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Unlock Route 2</t>
+          <t>Unlock Liberty Garden</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Extra Challenge E$3</t>
+          <t>Extra Challenge E$1</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Catch 10 Pokemon in Route 2</t>
+          <t>Complete Challenge 35</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Unlock Route 3</t>
+          <t>Unlock Route 1</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
+          <t>Extra Challenge E$2</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Catch 10 Pokemon in Route 1</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Unlock Route 2</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Extra Challenge E$3</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Catch 10 Pokemon in Route 2</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Unlock Route 3</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
           <t>Extra Challenge E$4</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B59" t="inlineStr">
         <is>
           <t>Catch 10 Pokemon in Route 3</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Unlock Nuvema Town</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Extra Challenge E$5</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Catch 10 Pokemon in Nuvema Town</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Unlock Abundant Shrine Depths</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Final Extra Challenge</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Complete Extra Challenge C$5, D$5, and E$5</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Unlock N's Castle</t>
         </is>
       </c>
     </row>
@@ -8070,7 +8398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D137"/>
+  <dimension ref="A1:D127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8098,34 +8426,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Victini</t>
+          <t>Servine</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Psychic / Fire</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Servine</t>
+          <t>Pignite</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Fire / Fighting</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8142,7 +8470,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Pignite</t>
+          <t>Emboar</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -8164,12 +8492,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Emboar</t>
+          <t>Dewott</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Fire / Fighting</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -8186,7 +8514,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Dewott</t>
+          <t>Samurott</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -8208,12 +8536,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Samurott</t>
+          <t>Unfezant</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Normal / Flying</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -8230,12 +8558,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Unfezant</t>
+          <t>Swadloon</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Normal / Flying</t>
+          <t>Bug / Grass</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -8252,7 +8580,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Swadloon</t>
+          <t>Leavanny</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -8274,12 +8602,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Leavanny</t>
+          <t>Sunflora</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bug / Grass</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -8296,12 +8624,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sunflora</t>
+          <t>Herdier</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -8318,7 +8646,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Herdier</t>
+          <t>Stoutland</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -8340,12 +8668,12 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Stoutland</t>
+          <t>Flaaffy</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -8362,7 +8690,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Flaaffy</t>
+          <t>Ampharos</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -8384,12 +8712,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Ampharos</t>
+          <t>Azumarill</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Water / Fairy</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -8406,12 +8734,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Azumarill</t>
+          <t>Lucario</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Water / Fairy</t>
+          <t>Fighting / Steel</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -8428,12 +8756,12 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Lucario</t>
+          <t>Simisage</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Fighting / Steel</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -8450,12 +8778,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Simisage</t>
+          <t>Simisear</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -8472,12 +8800,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Simisear</t>
+          <t>Simipour</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -8494,12 +8822,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Simipour</t>
+          <t>Whirlipede</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Bug / Poison</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -8516,7 +8844,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Whirlipede</t>
+          <t>Scolipede</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -8538,12 +8866,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Scolipede</t>
+          <t>Weezing</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Bug / Poison</t>
+          <t>Poison</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -8560,12 +8888,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Weezing</t>
+          <t>Magneton</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Poison</t>
+          <t>Electric / Steel</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -8582,7 +8910,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Magneton</t>
+          <t>Magnezone</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -8604,12 +8932,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Magnezone</t>
+          <t>Arcanine</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Electric / Steel</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -8626,7 +8954,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Arcanine</t>
+          <t>Magmar</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -8648,7 +8976,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Magmar</t>
+          <t>Magmortar</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -8670,12 +8998,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Magmortar</t>
+          <t>Electabuzz</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -8692,7 +9020,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Electabuzz</t>
+          <t>Electivire</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -8714,12 +9042,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Electivire</t>
+          <t>Crobat</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Poison / Flying</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -8736,12 +9064,12 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Crobat</t>
+          <t>Swoobat</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Poison / Flying</t>
+          <t>Psychic / Flying</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -8758,12 +9086,12 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Swoobat</t>
+          <t>Gigalith</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Psychic / Flying</t>
+          <t>Rock</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -8780,12 +9108,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Gigalith</t>
+          <t>Steelix</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Rock</t>
+          <t>Steel / Ground</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -8802,12 +9130,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Steelix</t>
+          <t>Conkeldurr</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Steel / Ground</t>
+          <t>Fighting</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -8824,12 +9152,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Conkeldurr</t>
+          <t>Musharna</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Fighting</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -8846,12 +9174,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Musharna</t>
+          <t>Clefable</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Fairy</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -8868,12 +9196,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Clefable</t>
+          <t>Vaporeon</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fairy</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -8890,12 +9218,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Vaporeon</t>
+          <t>Jolteon</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -8912,12 +9240,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Jolteon</t>
+          <t>Flareon</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -8934,12 +9262,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Flareon</t>
+          <t>Espeon</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -8956,12 +9284,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Espeon</t>
+          <t>Umbreon</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Dark</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -8978,12 +9306,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Umbreon</t>
+          <t>Leafeon</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Dark</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -9000,12 +9328,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Leafeon</t>
+          <t>Glaceon</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -9022,12 +9350,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Glaceon</t>
+          <t>Krokorok</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Ground / Dark</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -9044,7 +9372,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Krokorok</t>
+          <t>Krookodile</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -9066,66 +9394,66 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Krookodile</t>
+          <t>Darmanitan</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Ground / Dark</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Darmanitan</t>
+          <t>Cinccino</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Cinccino</t>
+          <t>Vullaby</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Dark / Flying</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -9528,7 +9856,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Aggron</t>
+          <t>Aron</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -9538,41 +9866,41 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Baltoy</t>
+          <t>Aggron</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Ground / Psychic</t>
+          <t>Steel / Rock</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Claydol</t>
+          <t>Baltoy</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -9594,78 +9922,78 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Volcarona</t>
+          <t>Claydol</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Bug / Fire</t>
+          <t>Ground / Psychic</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Galvantula</t>
+          <t>Larvesta</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Bug / Electric</t>
+          <t>Bug / Fire</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Ferrothorn</t>
+          <t>Volcarona</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Grass / Steel</t>
+          <t>Bug / Fire</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Eelektross</t>
+          <t>Galvantula</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Electric</t>
+          <t>Bug / Electric</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -9682,12 +10010,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Fraxure</t>
+          <t>Ferrothorn</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dragon</t>
+          <t>Grass / Steel</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -9704,12 +10032,12 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Haxorus</t>
+          <t>Eelektross</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Dragon</t>
+          <t>Electric</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -9726,100 +10054,100 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Zangoose</t>
+          <t>Fraxure</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Dragon</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Seviper</t>
+          <t>Haxorus</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Poison</t>
+          <t>Dragon</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Beheeyem</t>
+          <t>Zangoose</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Lampent</t>
+          <t>Seviper</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Ghost / Fire</t>
+          <t>Poison</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Chandelure</t>
+          <t>Beheeyem</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Ghost / Fire</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -9836,12 +10164,12 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Beartic</t>
+          <t>Lampent</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Ghost / Fire</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -9858,56 +10186,56 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Tornadus</t>
+          <t>Chandelure</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Ghost / Fire</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Thundurus</t>
+          <t>Beartic</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Landorus</t>
+          <t>Skorupi</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Poison / Bug</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -9924,12 +10252,12 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Skorupi</t>
+          <t>Drapion</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Poison / Bug</t>
+          <t>Poison / Dark</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -9946,12 +10274,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Drapion</t>
+          <t>Numel</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Poison / Dark</t>
+          <t>Fire / Ground</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -9968,56 +10296,56 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Numel</t>
+          <t>Grumpig</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Fire / Ground</t>
+          <t>Psychic</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Grumpig</t>
+          <t>Drifloon</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Psychic</t>
+          <t>Ghost / Flying</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Drifloon</t>
+          <t>Shuppet</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Ghost / Flying</t>
+          <t>Ghost</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -10034,12 +10362,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Shuppet</t>
+          <t>Lunatone</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Ghost</t>
+          <t>Rock / Psychic</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -10056,7 +10384,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Lunatone</t>
+          <t>Solrock</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -10078,34 +10406,34 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Solrock</t>
+          <t>Tangrowth</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Rock / Psychic</t>
+          <t>Grass</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Tangrowth</t>
+          <t>Mienshao</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Grass</t>
+          <t>Fighting</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -10122,12 +10450,12 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Mienshao</t>
+          <t>Gliscor</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Fighting</t>
+          <t>Ground / Flying</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -10144,12 +10472,12 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Gliscor</t>
+          <t>Bisharp</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Ground / Flying</t>
+          <t>Dark / Steel</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -10166,12 +10494,12 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>Bisharp</t>
+          <t>Seismitoad</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Dark / Steel</t>
+          <t>Water / Ground</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -10188,12 +10516,12 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Cobalion</t>
+          <t>Shuckle</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Steel / Fighting</t>
+          <t>Bug / Rock</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -10210,56 +10538,56 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Terrakion</t>
+          <t>Mantine</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Rock / Fighting</t>
+          <t>Water / Flying</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>Virizion</t>
+          <t>Octillery</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Grass / Fighting</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Seismitoad</t>
+          <t>Starmie</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Water / Ground</t>
+          <t>Water / Psychic</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -10276,12 +10604,12 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Shuckle</t>
+          <t>Wailmer</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Bug / Rock</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -10298,34 +10626,34 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Mantine</t>
+          <t>Wailord</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Water / Flying</t>
+          <t>Water</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Octillery</t>
+          <t>Sealeo</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Ice / Water</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -10342,12 +10670,12 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Starmie</t>
+          <t>Walrein</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Water / Psychic</t>
+          <t>Ice / Water</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -10364,56 +10692,56 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>Wailmer</t>
+          <t>Ninetales</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Fire</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Wailord</t>
+          <t>Weavile</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Dark / Ice</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Sealeo</t>
+          <t>Vanillish</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Ice / Water</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -10430,12 +10758,12 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Walrein</t>
+          <t>Vanilluxe</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Ice / Water</t>
+          <t>Ice</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -10452,12 +10780,12 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Ninetales</t>
+          <t>Mamoswine</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Fire</t>
+          <t>Ice / Ground</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -10474,12 +10802,12 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Weavile</t>
+          <t>Metagross</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Dark / Ice</t>
+          <t>Steel / Psychic</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -10496,12 +10824,12 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Vanillish</t>
+          <t>Dewgong</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Water / Ice</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -10518,12 +10846,12 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Vanilluxe</t>
+          <t>Golurk</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Ice</t>
+          <t>Ground / Ghost</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -10540,12 +10868,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Mamoswine</t>
+          <t>Zweilous</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Ice / Ground</t>
+          <t>Dark / Dragon</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -10562,12 +10890,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Metagross</t>
+          <t>Hydreigon</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Steel / Psychic</t>
+          <t>Dark / Dragon</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -10584,78 +10912,78 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Dewgong</t>
+          <t>Slakoth</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Water / Ice</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Golurk</t>
+          <t>Vigoroth</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Ground / Ghost</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Zweilous</t>
+          <t>Slaking</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Dark / Dragon</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Hydreigon</t>
+          <t>Crawdaunt</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Dark / Dragon</t>
+          <t>Water / Dark</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -10672,51 +11000,51 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Slakoth</t>
+          <t>Jigglypuff</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Normal / Fairy</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Vigoroth</t>
+          <t>Wigglytuff</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Normal / Fairy</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Slaking</t>
+          <t>Lickitung</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -10738,34 +11066,34 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Crawdaunt</t>
+          <t>Lickilicky</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Water / Dark</t>
+          <t>Normal</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Jigglypuff</t>
+          <t>Yanmega</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Normal / Fairy</t>
+          <t>Bug / Flying</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -10782,56 +11110,56 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Wigglytuff</t>
+          <t>Tropius</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Normal / Fairy</t>
+          <t>Grass / Flying</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Suggest: Route 1</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Lickitung</t>
+          <t>Toxicroak</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Poison / Fighting</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Suggest: Route 1</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Lickilicky</t>
+          <t>Larvitar</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Normal</t>
+          <t>Rock / Ground</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -10848,12 +11176,12 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Yanmega</t>
+          <t>Tyranitar</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Bug / Flying</t>
+          <t>Rock / Dark</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -10864,226 +11192,6 @@
       <c r="D127" t="inlineStr">
         <is>
           <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="128">
-      <c r="A128" t="inlineStr">
-        <is>
-          <t>Tropius</t>
-        </is>
-      </c>
-      <c r="B128" t="inlineStr">
-        <is>
-          <t>Grass / Flying</t>
-        </is>
-      </c>
-      <c r="C128" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D128" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>Toxicroak</t>
-        </is>
-      </c>
-      <c r="B129" t="inlineStr">
-        <is>
-          <t>Poison / Fighting</t>
-        </is>
-      </c>
-      <c r="C129" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D129" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" t="inlineStr">
-        <is>
-          <t>Larvitar</t>
-        </is>
-      </c>
-      <c r="B130" t="inlineStr">
-        <is>
-          <t>Rock / Ground</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D130" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" t="inlineStr">
-        <is>
-          <t>Tyranitar</t>
-        </is>
-      </c>
-      <c r="B131" t="inlineStr">
-        <is>
-          <t>Rock / Dark</t>
-        </is>
-      </c>
-      <c r="C131" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D131" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>Reshiram</t>
-        </is>
-      </c>
-      <c r="B132" t="inlineStr">
-        <is>
-          <t>Dragon / Fire</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D132" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="133">
-      <c r="A133" t="inlineStr">
-        <is>
-          <t>Zekrom</t>
-        </is>
-      </c>
-      <c r="B133" t="inlineStr">
-        <is>
-          <t>Dragon / Electric</t>
-        </is>
-      </c>
-      <c r="C133" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D133" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="134">
-      <c r="A134" t="inlineStr">
-        <is>
-          <t>Kyurem</t>
-        </is>
-      </c>
-      <c r="B134" t="inlineStr">
-        <is>
-          <t>Dragon / Ice</t>
-        </is>
-      </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D134" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="135">
-      <c r="A135" t="inlineStr">
-        <is>
-          <t>Keldeo</t>
-        </is>
-      </c>
-      <c r="B135" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C135" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D135" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="136">
-      <c r="A136" t="inlineStr">
-        <is>
-          <t>Meloetta</t>
-        </is>
-      </c>
-      <c r="B136" t="inlineStr">
-        <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="C136" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D136" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-    </row>
-    <row r="137">
-      <c r="A137" t="inlineStr">
-        <is>
-          <t>Genesect</t>
-        </is>
-      </c>
-      <c r="B137" t="inlineStr">
-        <is>
-          <t>Bug / Steel</t>
-        </is>
-      </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>Suggest: Route 1</t>
-        </is>
-      </c>
-      <c r="D137" t="inlineStr">
-        <is>
-          <t>No</t>
         </is>
       </c>
     </row>

</xml_diff>